<commit_message>
Finished Training for Pipeline
</commit_message>
<xml_diff>
--- a/HalfCache/OverallStatsCacheHalf-Noboot.xlsx
+++ b/HalfCache/OverallStatsCacheHalf-Noboot.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexb\OneDrive\Documents\Thesis\HalfCache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9168156B-51F0-4A89-B261-4DB2DA17EE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E979FC4B-5A51-406A-BDEF-451F559C1D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="1830" windowWidth="38640" windowHeight="21120" xr2:uid="{84A3B88E-B226-40B3-A64E-0FDCC502A4B5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{84A3B88E-B226-40B3-A64E-0FDCC502A4B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
   <si>
     <t>HalfCache</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>Nu: 0.5, Gamma: 0.7</t>
+  </si>
+  <si>
+    <t>Accuracy (%)</t>
   </si>
 </sst>
 </file>
@@ -509,7 +512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{652EE7E4-9A64-4328-97BF-22E9AA604A6A}">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.36328125" customWidth="1"/>
@@ -572,10 +575,10 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3">
         <v>18</v>
@@ -585,11 +588,11 @@
       </c>
       <c r="H3">
         <f>(C3)/(C3+D3)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I3">
         <f>C3/(C3+E3)</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J3">
         <f>(2*(H3*I3))/(H3+I3)</f>
@@ -597,7 +600,7 @@
       </c>
       <c r="K3">
         <f>F3/(F3+D3)</f>
-        <v>0.94736842105263153</v>
+        <v>1</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -617,10 +620,10 @@
         <v>3</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4">
         <v>45</v>
@@ -630,11 +633,11 @@
       </c>
       <c r="H4">
         <f t="shared" ref="H4:H13" si="0">(C4)/(C4+D4)</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="I4">
         <f t="shared" ref="I4:I13" si="1">C4/(C4+E4)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="J4">
         <f t="shared" ref="J4:J13" si="2">(2*(H4*I4))/(H4+I4)</f>
@@ -642,7 +645,7 @@
       </c>
       <c r="K4">
         <f t="shared" ref="K4:K13" si="3">F4/(F4+D4)</f>
-        <v>0.97826086956521741</v>
+        <v>1</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -662,10 +665,10 @@
         <v>1</v>
       </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
         <v>4</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
       </c>
       <c r="F5">
         <v>44</v>
@@ -675,11 +678,11 @@
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I5">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="J5">
         <f t="shared" si="2"/>
@@ -687,7 +690,7 @@
       </c>
       <c r="K5">
         <f t="shared" si="3"/>
-        <v>0.91666666666666663</v>
+        <v>1</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -707,10 +710,10 @@
         <v>22</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6">
         <v>1210</v>
@@ -720,11 +723,11 @@
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
-        <v>0.95652173913043481</v>
+        <v>1</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.95652173913043481</v>
       </c>
       <c r="J6">
         <f t="shared" si="2"/>
@@ -732,7 +735,7 @@
       </c>
       <c r="K6">
         <f t="shared" si="3"/>
-        <v>0.9991742361684558</v>
+        <v>1</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -752,10 +755,10 @@
         <v>1</v>
       </c>
       <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
         <v>3</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
       </c>
       <c r="F7">
         <v>133</v>
@@ -765,11 +768,11 @@
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="I7">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="J7">
         <f t="shared" si="2"/>
@@ -777,7 +780,7 @@
       </c>
       <c r="K7">
         <f t="shared" si="3"/>
-        <v>0.9779411764705882</v>
+        <v>1</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -797,10 +800,10 @@
         <v>1</v>
       </c>
       <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
         <v>15</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
       </c>
       <c r="F8">
         <v>207</v>
@@ -810,11 +813,11 @@
       </c>
       <c r="H8">
         <f t="shared" si="0"/>
-        <v>6.25E-2</v>
+        <v>1</v>
       </c>
       <c r="I8">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>6.25E-2</v>
       </c>
       <c r="J8">
         <f t="shared" si="2"/>
@@ -822,7 +825,7 @@
       </c>
       <c r="K8">
         <f t="shared" si="3"/>
-        <v>0.93243243243243246</v>
+        <v>1</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -842,10 +845,10 @@
         <v>0</v>
       </c>
       <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
         <v>4</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
       </c>
       <c r="F9">
         <v>36</v>
@@ -853,13 +856,13 @@
       <c r="G9">
         <v>90</v>
       </c>
-      <c r="H9">
+      <c r="H9" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I9" t="e">
-        <f>C9/(C9+E9)</f>
         <v>#DIV/0!</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="J9" t="e">
         <f>(2*(H9*I9))/(H9+I9)</f>
@@ -867,7 +870,7 @@
       </c>
       <c r="K9">
         <f t="shared" si="3"/>
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -887,10 +890,10 @@
         <v>22</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10">
         <v>116</v>
@@ -900,11 +903,11 @@
       </c>
       <c r="H10">
         <f t="shared" si="0"/>
-        <v>0.95652173913043481</v>
+        <v>1</v>
       </c>
       <c r="I10">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.95652173913043481</v>
       </c>
       <c r="J10">
         <f t="shared" si="2"/>
@@ -912,7 +915,7 @@
       </c>
       <c r="K10">
         <f t="shared" si="3"/>
-        <v>0.99145299145299148</v>
+        <v>1</v>
       </c>
       <c r="L10">
         <v>10</v>
@@ -932,10 +935,10 @@
         <v>3</v>
       </c>
       <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
         <v>2</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
       </c>
       <c r="F11">
         <v>47</v>
@@ -945,11 +948,11 @@
       </c>
       <c r="H11">
         <f t="shared" si="0"/>
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I11">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="J11">
         <f t="shared" si="2"/>
@@ -957,7 +960,7 @@
       </c>
       <c r="K11">
         <f t="shared" si="3"/>
-        <v>0.95918367346938771</v>
+        <v>1</v>
       </c>
       <c r="L11">
         <v>10</v>
@@ -977,10 +980,10 @@
         <v>1</v>
       </c>
       <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
         <v>11</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
       </c>
       <c r="F12">
         <v>129</v>
@@ -990,19 +993,19 @@
       </c>
       <c r="H12">
         <f t="shared" si="0"/>
-        <v>8.3333333333333329E-2</v>
+        <v>1</v>
       </c>
       <c r="I12">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="J12">
-        <f t="shared" si="2"/>
+        <f>(2*(H12*I12))/(H12+I12)</f>
         <v>0.15384615384615385</v>
       </c>
       <c r="K12">
         <f t="shared" si="3"/>
-        <v>0.92142857142857137</v>
+        <v>1</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1022,10 +1025,10 @@
         <v>464</v>
       </c>
       <c r="D13">
+        <v>47</v>
+      </c>
+      <c r="E13">
         <v>38</v>
-      </c>
-      <c r="E13">
-        <v>47</v>
       </c>
       <c r="F13">
         <v>4971</v>
@@ -1035,11 +1038,11 @@
       </c>
       <c r="H13">
         <f t="shared" si="0"/>
-        <v>0.92430278884462147</v>
+        <v>0.90802348336594907</v>
       </c>
       <c r="I13">
         <f t="shared" si="1"/>
-        <v>0.90802348336594907</v>
+        <v>0.92430278884462147</v>
       </c>
       <c r="J13">
         <f t="shared" si="2"/>
@@ -1047,13 +1050,200 @@
       </c>
       <c r="K13">
         <f t="shared" si="3"/>
-        <v>0.99241365542024351</v>
+        <v>0.99063371861299321</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
         <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25">
+        <v>97.959183673469298</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>0.75</v>
+      </c>
+      <c r="E25">
+        <v>0.8571428571428571</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26">
+        <v>86.274509800000004</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>0.2</v>
+      </c>
+      <c r="E26">
+        <v>0.33333333333333337</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27">
+        <v>99.918896999188902</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>0.95652173913043481</v>
+      </c>
+      <c r="E27">
+        <v>0.97777777777777775</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28">
+        <v>97.810218978102199</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>0.25</v>
+      </c>
+      <c r="E28">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29">
+        <v>93.273542600896803</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29">
+        <v>6.25E-2</v>
+      </c>
+      <c r="E29">
+        <v>0.11764705882352941</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30">
+        <v>90</v>
+      </c>
+      <c r="C30" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="e">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31">
+        <v>98.353909470000005</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>0.95652173913043481</v>
+      </c>
+      <c r="E31">
+        <v>0.97777777777777775</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32">
+        <v>96.153846153846104</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32">
+        <v>0.6</v>
+      </c>
+      <c r="E32">
+        <v>0.74999999999999989</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33">
+        <v>92.1985815602836</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+      <c r="D33">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E33">
+        <v>0.15384615384615385</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34">
+        <v>98.460144929999998</v>
+      </c>
+      <c r="C34">
+        <v>0.90802348336594907</v>
+      </c>
+      <c r="D34">
+        <v>0.92430278884462147</v>
+      </c>
+      <c r="E34">
+        <v>0.91609081934846981</v>
       </c>
     </row>
   </sheetData>

</xml_diff>